<commit_message>
Fill Europa League 2026/27 matchday 1 results
18 results from UEFA's match data. The Conference League starts on
15 October. fill_from_uefa.py now repeats its name-inference pass until
nothing new is found, which paired the last remaining row.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/europa-league/uefa-results-2026-27.xlsx
+++ b/europa-league/uefa-results-2026-27.xlsx
@@ -785,8 +785,12 @@
           <t>Sparta Prague</t>
         </is>
       </c>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
+      <c r="E2" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>4</v>
+      </c>
       <c r="G2" s="9" t="n"/>
     </row>
     <row r="3">
@@ -810,8 +814,12 @@
           <t>Celta Vigo</t>
         </is>
       </c>
-      <c r="E3" s="9" t="n"/>
-      <c r="F3" s="9" t="n"/>
+      <c r="E3" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G3" s="9" t="n"/>
     </row>
     <row r="4">
@@ -835,8 +843,12 @@
           <t>Benfica</t>
         </is>
       </c>
-      <c r="E4" s="9" t="n"/>
-      <c r="F4" s="9" t="n"/>
+      <c r="E4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G4" s="9" t="n"/>
     </row>
     <row r="5">
@@ -860,8 +872,12 @@
           <t>Celje</t>
         </is>
       </c>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
+      <c r="E5" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G5" s="9" t="n"/>
     </row>
     <row r="6">
@@ -885,8 +901,12 @@
           <t>Dinamo Zagreb</t>
         </is>
       </c>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G6" s="9" t="n"/>
     </row>
     <row r="7">
@@ -910,8 +930,12 @@
           <t>Jagiellonia Białystok</t>
         </is>
       </c>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
+      <c r="E7" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G7" s="9" t="n"/>
     </row>
     <row r="8">
@@ -935,8 +959,12 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
+      <c r="E8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G8" s="9" t="n"/>
     </row>
     <row r="9">
@@ -960,8 +988,12 @@
           <t>Rennes</t>
         </is>
       </c>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
+      <c r="E9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G9" s="9" t="n"/>
     </row>
     <row r="10">
@@ -985,8 +1017,12 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
+      <c r="E10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G10" s="9" t="n"/>
     </row>
     <row r="11">
@@ -1010,8 +1046,12 @@
           <t>TSG Hoffenheim</t>
         </is>
       </c>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
+      <c r="E11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G11" s="9" t="n"/>
     </row>
     <row r="12">
@@ -1035,8 +1075,12 @@
           <t>Red Bull Salzburg</t>
         </is>
       </c>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
+      <c r="E12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G12" s="9" t="n"/>
     </row>
     <row r="13">
@@ -1060,8 +1104,12 @@
           <t>Marseille</t>
         </is>
       </c>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
+      <c r="E13" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G13" s="9" t="n"/>
     </row>
     <row r="14">
@@ -1085,8 +1133,12 @@
           <t>Ferencváros</t>
         </is>
       </c>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
+      <c r="E14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="G14" s="9" t="n"/>
     </row>
     <row r="15">
@@ -1110,8 +1162,12 @@
           <t>Lech Poznań</t>
         </is>
       </c>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="9" t="n"/>
+      <c r="E15" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G15" s="9" t="n"/>
     </row>
     <row r="16">
@@ -1135,8 +1191,12 @@
           <t>Union Saint-Gilloise</t>
         </is>
       </c>
-      <c r="E16" s="9" t="n"/>
-      <c r="F16" s="9" t="n"/>
+      <c r="E16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="G16" s="9" t="n"/>
     </row>
     <row r="17">
@@ -1160,8 +1220,12 @@
           <t>NEC</t>
         </is>
       </c>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="9" t="n"/>
+      <c r="E17" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G17" s="9" t="n"/>
     </row>
     <row r="18">
@@ -1185,8 +1249,12 @@
           <t>Torreense</t>
         </is>
       </c>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9" t="n"/>
+      <c r="E18" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G18" s="9" t="n"/>
     </row>
     <row r="19">
@@ -1210,8 +1278,12 @@
           <t>Bournemouth</t>
         </is>
       </c>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="n"/>
+      <c r="E19" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G19" s="9" t="n"/>
     </row>
     <row r="20">

</xml_diff>